<commit_message>
Update root-level Excel report for 28-07-2026 with 3 businesses found
</commit_message>
<xml_diff>
--- a/דוח נכסים לתאריך:28-07-2026.xlsx
+++ b/דוח נכסים לתאריך:28-07-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="דוח עסקים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="דוח נכסים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,6 +35,12 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -46,19 +52,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
-        <bgColor rgb="00D6E4F0"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -96,7 +99,13 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -464,16 +473,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -513,20 +522,20 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>חווה ש. נתן</t>
+          <t>לשון זהב מאנגלית לעברית</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>הפלמח 32, ירושלים</t>
+          <t>הקבלן 1, ירושלים</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>מרצים</t>
+          <t>שירותי תרגום</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -534,57 +543,57 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/29715390/32150/</t>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80011462/51870/</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>יצחק כהן</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>הפלמח 49, ירושלים</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>מנעולנים</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>עו"ד מלכן אברהם</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>הקבלן 15, ירושלים</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>עורך דין - משפט אזרחי ✅</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80149703/29970/</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80284569/9010104/</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
     </row>
-    <row r="4" ht="20" customHeight="1">
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>בתאל גולדברג - מטפלת רגשית</t>
+          <t>איגוד רשויות הכשרות מאגר מידע</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>הפרטיזנים 304, ירושלים</t>
+          <t>הקבלן 15, ירושלים</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>ייעוץ וטיפול רגשי</t>
+          <t>יועצי מזון / כשרות</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -592,305 +601,20 @@
           <t>גבוה</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80283036/19745/</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/35664450/24870/</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>פרלה נמרובסקי - קוסמטיקאית</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>הפרטיזנים 304, ירושלים</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>קוסמטיקאיות</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80247737/43860/</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>גוני שילון רם</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>הצבעוני 1, ירושלים</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>תיקשור</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/70237570/40030028/</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>ארצנו תורס בע"מ</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>הצדיק משטפנשט 24, ירושלים</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>טיולים מאורגנים</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/39252600/33600/</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>מנת טובי</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>הצדיק משטפנשט 41, ירושלים</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>מדריכי ספורט וכושר</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80244104/22570/</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>תור אופטיקה</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>הצדיק משטפנשט 43, ירושלים</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>אופטיקאים</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80143688/1560/</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>אלי כץ</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>הצבר 202, ירושלים</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>רפדים</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/18506680/47520/</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>בר לב ביני</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>הצפירה 12, ירושלים</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>עורכי דין</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80016281/38010/</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>מינימרקט מעלומי</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>הצפירה 12, ירושלים</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>סופרמרקטים ומכולות</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/9556740/35760/</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>ידיד אליהו</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>הצפירה 24, ירושלים</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>קבלני בניין</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/6064910/43470/</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>טכנו עמליה - לוי עובדיה</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>הצפירה 25, ירושלים</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>עיבוד שיש</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/4154630/48810/</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>